<commit_message>
now check cell reference consistency. Import styles export
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/SetCellColorOut.xlsx
+++ b/3-Dev/DevApp/Files/SetCellColorOut.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E4C2215-20B3-4139-B2DD-2F9E801C024D}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F328B5E8-7FB8-4B0E-B017-4E5B9A35B2E8}"/>
   <bookViews>
-    <workbookView xWindow="3615" yWindow="6180" windowWidth="19065" windowHeight="9735" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
+    <workbookView xWindow="17055" yWindow="2415" windowWidth="10980" windowHeight="13395" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>cell</t>
   </si>
@@ -63,12 +63,6 @@
   </si>
   <si>
     <t>null, set to green</t>
-  </si>
-  <si>
-    <t>nofill, border, set to orange</t>
-  </si>
-  <si>
-    <t>later</t>
   </si>
   <si>
     <t>green, to to red</t>
@@ -144,6 +138,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C34316-5981-45DA-B1A5-D1338D5ADA96}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
@@ -493,7 +491,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -501,7 +499,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -512,7 +510,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -520,113 +518,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>